<commit_message>
Escáner 2 HEO: Excel con «Ventas» (caídas 30 d), caja de compra FBA con 'yes' y marca no mirada como diferencia de criterio (encargo D)
Hoja Análisis: 'Rank actual' pasa a 'Ventas' (caídas de 30 días; 0 es 0, sin dato vacío); fuera Rank 90d, Vendidos/mes, Nº ofertas y Promo activa (27 columnas). Desvíos deliberados sobre la copia del viejo en escaner2_desvios.py, aplicados al regenerar. Beneficio, ROI y Margen sin cambios (5.370 celdas comparadas con datos reales). Lector de Keepa del escáner 2: 'yes' = FBA. Comparación: la marca no mirada en la pasada pasa a diferencia de criterio. No toca el escáner viejo ni la elección de puerta y mejor país. Decisión de Fernando del 28-sep-2026.
</commit_message>
<xml_diff>
--- a/excel_referencia_escaner2.xlsx
+++ b/excel_referencia_escaner2.xlsx
@@ -203,40 +203,36 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_Analisis" displayName="T_Analisis" ref="A1:AE17" headerRowCount="1">
-  <autoFilter ref="A1:AE17"/>
-  <tableColumns count="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_Analisis" displayName="T_Analisis" ref="A1:AA17" headerRowCount="1">
+  <autoFilter ref="A1:AA17"/>
+  <tableColumns count="27">
     <tableColumn id="1" name="Nombre"/>
     <tableColumn id="2" name="EAN"/>
     <tableColumn id="3" name="ASIN"/>
     <tableColumn id="4" name="Marca"/>
     <tableColumn id="5" name="PA (€)"/>
     <tableColumn id="6" name="País"/>
-    <tableColumn id="7" name="Rank actual"/>
-    <tableColumn id="8" name="Rank 90d"/>
-    <tableColumn id="9" name="Vendidos/mes"/>
-    <tableColumn id="10" name="Precio venta (€)"/>
-    <tableColumn id="11" name="Canal BB"/>
-    <tableColumn id="12" name="Nº ofertas"/>
-    <tableColumn id="13" name="% Comisión"/>
-    <tableColumn id="14" name="Com. Amazon (€)"/>
-    <tableColumn id="15" name="Fee Logística (€)"/>
-    <tableColumn id="16" name="Almacén (€)"/>
-    <tableColumn id="17" name="Promo activa"/>
-    <tableColumn id="18" name="Beneficio (€)"/>
-    <tableColumn id="19" name="ROI"/>
-    <tableColumn id="20" name="Margen"/>
-    <tableColumn id="21" name="Decisión"/>
-    <tableColumn id="22" name="En mi BD"/>
-    <tableColumn id="23" name="EAN ambiguo"/>
-    <tableColumn id="24" name="Amazon (título)"/>
-    <tableColumn id="25" name="Coincide"/>
-    <tableColumn id="26" name="Cotejo"/>
-    <tableColumn id="27" name="Cotejo (detalle)"/>
-    <tableColumn id="28" name="Coherencia caja"/>
-    <tableColumn id="29" name="OcioStock"/>
-    <tableColumn id="30" name="ISD s/ Fee Log. (€)"/>
-    <tableColumn id="31" name="Origen IVA"/>
+    <tableColumn id="7" name="Ventas"/>
+    <tableColumn id="8" name="Precio venta (€)"/>
+    <tableColumn id="9" name="Canal BB"/>
+    <tableColumn id="10" name="% Comisión"/>
+    <tableColumn id="11" name="Com. Amazon (€)"/>
+    <tableColumn id="12" name="Fee Logística (€)"/>
+    <tableColumn id="13" name="Almacén (€)"/>
+    <tableColumn id="14" name="Beneficio (€)"/>
+    <tableColumn id="15" name="ROI"/>
+    <tableColumn id="16" name="Margen"/>
+    <tableColumn id="17" name="Decisión"/>
+    <tableColumn id="18" name="En mi BD"/>
+    <tableColumn id="19" name="EAN ambiguo"/>
+    <tableColumn id="20" name="Amazon (título)"/>
+    <tableColumn id="21" name="Coincide"/>
+    <tableColumn id="22" name="Cotejo"/>
+    <tableColumn id="23" name="Cotejo (detalle)"/>
+    <tableColumn id="24" name="Coherencia caja"/>
+    <tableColumn id="25" name="OcioStock"/>
+    <tableColumn id="26" name="ISD s/ Fee Log. (€)"/>
+    <tableColumn id="27" name="Origen IVA"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -531,23 +527,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AA17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="50" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="16" customWidth="1" min="26" max="26"/>
-    <col width="46" customWidth="1" min="27" max="27"/>
-    <col width="46" customWidth="1" min="28" max="28"/>
-    <col width="13" customWidth="1" min="29" max="29"/>
-    <col width="17" customWidth="1" min="30" max="30"/>
-    <col width="14" customWidth="1" min="31" max="31"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="50" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="46" customWidth="1" min="23" max="23"/>
+    <col width="46" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="17" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -583,125 +579,105 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Rank actual</t>
+          <t>Ventas</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Rank 90d</t>
+          <t>Precio venta (€)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Vendidos/mes</t>
+          <t>Canal BB</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Precio venta (€)</t>
+          <t>% Comisión</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Canal BB</t>
+          <t>Com. Amazon (€)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Nº ofertas</t>
+          <t>Fee Logística (€)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>% Comisión</t>
+          <t>Almacén (€)</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Com. Amazon (€)</t>
+          <t>Beneficio (€)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Fee Logística (€)</t>
+          <t>ROI</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Almacén (€)</t>
+          <t>Margen</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Promo activa</t>
+          <t>Decisión</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Beneficio (€)</t>
+          <t>En mi BD</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>ROI</t>
+          <t>EAN ambiguo</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Margen</t>
+          <t>Amazon (título)</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Coincide</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>En mi BD</t>
+          <t>Cotejo</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>EAN ambiguo</t>
+          <t>Cotejo (detalle)</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Amazon (título)</t>
+          <t>Coherencia caja</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Coincide</t>
+          <t>OcioStock</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>Cotejo</t>
+          <t>ISD s/ Fee Log. (€)</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>Cotejo (detalle)</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Coherencia caja</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>OcioStock</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>ISD s/ Fee Log. (€)</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Origen IVA</t>
         </is>
@@ -737,91 +713,82 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2400</v>
-      </c>
-      <c r="I2" t="n">
-        <v>40</v>
-      </c>
-      <c r="J2" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="H2" s="3" t="n">
         <v>19.99</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>BB-FBA</t>
         </is>
       </c>
-      <c r="L2" t="n">
-        <v>7</v>
-      </c>
-      <c r="M2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>0.1545</v>
       </c>
+      <c r="K2" s="3">
+        <f>H2*J2+Z2</f>
+        <v/>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N2" s="3">
-        <f>J2*M2+AD2</f>
+        <f>(H2/1.1)-E2-K2-L2-M2</f>
         <v/>
       </c>
-      <c r="O2" s="3" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="P2" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R2" s="3">
-        <f>(J2/1.1)-E2-N2-O2-P2</f>
+      <c r="O2" s="5">
+        <f>N2/E2</f>
         <v/>
       </c>
-      <c r="S2" s="5">
-        <f>R2/E2</f>
+      <c r="P2" s="5">
+        <f>N2/H2</f>
         <v/>
       </c>
-      <c r="T2" s="5">
-        <f>R2/J2</f>
-        <v/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>COMPRAR</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>OK Alm:3 FBA:5</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Titulo de prueba Alfa</t>
+        </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>COMPRAR</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>OK Alm:3 FBA:5</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>2/2 casan; entre esos, mejor rank (casa: alfa)</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Titulo de prueba Alfa</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="AA2" t="inlineStr">
-        <is>
-          <t>2/2 casan; entre esos, mejor rank (casa: alfa)</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE2" t="inlineStr">
         <is>
           <t>ficha</t>
         </is>
@@ -857,91 +824,82 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>3000</v>
-      </c>
-      <c r="H3" t="n">
-        <v>6000</v>
-      </c>
-      <c r="I3" t="n">
-        <v>40</v>
-      </c>
-      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3" t="n">
         <v>17.5</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>BB-FBA</t>
         </is>
       </c>
-      <c r="L3" t="n">
-        <v>7</v>
-      </c>
-      <c r="M3" s="4" t="n">
+      <c r="J3" s="4" t="n">
         <v>0.1545</v>
       </c>
+      <c r="K3" s="3">
+        <f>H3*J3+Z3</f>
+        <v/>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N3" s="3">
-        <f>J3*M3+AD3</f>
+        <f>(H3/1.22)-E3-K3-L3-M3</f>
         <v/>
       </c>
-      <c r="O3" s="3" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="P3" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R3" s="3">
-        <f>(J3/1.22)-E3-N3-O3-P3</f>
+      <c r="O3" s="5">
+        <f>N3/E3</f>
         <v/>
       </c>
-      <c r="S3" s="5">
-        <f>R3/E3</f>
+      <c r="P3" s="5">
+        <f>N3/H3</f>
         <v/>
       </c>
-      <c r="T3" s="5">
-        <f>R3/J3</f>
-        <v/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>VALORAR</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>OK Alm:3 FBA:5</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Titulo de prueba Alfa</t>
+        </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>VALORAR</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>OK Alm:3 FBA:5</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>2/2 casan; entre esos, mejor rank (casa: alfa)</t>
+        </is>
+      </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Titulo de prueba Alfa</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="AA3" t="inlineStr">
-        <is>
-          <t>2/2 casan; entre esos, mejor rank (casa: alfa)</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE3" t="inlineStr">
         <is>
           <t>general IT 22%</t>
         </is>
@@ -976,93 +934,81 @@
           <t>FR</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H4" t="n">
-        <v>100000</v>
-      </c>
-      <c r="I4" t="n">
-        <v>40</v>
-      </c>
-      <c r="J4" s="3" t="n">
+      <c r="H4" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>BB-FBA</t>
         </is>
       </c>
-      <c r="L4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>0.1545</v>
       </c>
+      <c r="K4" s="3">
+        <f>H4*J4+Z4</f>
+        <v/>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N4" s="3">
-        <f>J4*M4+AD4</f>
+        <f>(H4/1.2)-E4-K4-L4-M4</f>
         <v/>
       </c>
-      <c r="O4" s="3" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="P4" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R4" s="3">
-        <f>(J4/1.2)-E4-N4-O4-P4</f>
+      <c r="O4" s="5">
+        <f>N4/E4</f>
         <v/>
       </c>
-      <c r="S4" s="5">
-        <f>R4/E4</f>
+      <c r="P4" s="5">
+        <f>N4/H4</f>
         <v/>
       </c>
-      <c r="T4" s="5">
-        <f>R4/J4</f>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>NO COMPRAR</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>OK Alm:3 FBA:5</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Titulo de prueba Alfa</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>2/2 casan; entre esos, mejor rank (casa: alfa)</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" s="3">
+        <f>L4*0.03</f>
         <v/>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>NO COMPRAR</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>OK Alm:3 FBA:5</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>Titulo de prueba Alfa</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
       <c r="AA4" t="inlineStr">
-        <is>
-          <t>2/2 casan; entre esos, mejor rank (casa: alfa)</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" s="3">
-        <f>O4*0.03</f>
-        <v/>
-      </c>
-      <c r="AE4" t="inlineStr">
         <is>
           <t>general FR 20%</t>
         </is>
@@ -1097,68 +1043,65 @@
           <t>DE</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>40</v>
-      </c>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" t="inlineStr">
+      <c r="G5" t="n">
+        <v>12</v>
+      </c>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" t="inlineStr">
         <is>
           <t>BB-FBA</t>
         </is>
       </c>
-      <c r="L5" t="n">
-        <v>7</v>
-      </c>
-      <c r="M5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R5" s="3" t="n"/>
-      <c r="S5" s="5" t="n"/>
-      <c r="T5" s="5" t="n"/>
+      <c r="O5" s="5" t="n"/>
+      <c r="P5" s="5" t="n"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Sin datos</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>OK Alm:3 FBA:5</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Titulo de prueba Alfa</t>
+        </is>
+      </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Sin datos</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>OK Alm:3 FBA:5</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>2/2 casan; entre esos, mejor rank (casa: alfa)</t>
+        </is>
+      </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>Titulo de prueba Alfa</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="AA5" t="inlineStr">
-        <is>
-          <t>2/2 casan; entre esos, mejor rank (casa: alfa)</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE5" t="inlineStr">
         <is>
           <t>general DE 19%</t>
         </is>
@@ -1194,99 +1137,90 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>8000</v>
-      </c>
-      <c r="H6" t="n">
-        <v>16000</v>
-      </c>
-      <c r="I6" t="n">
-        <v>40</v>
-      </c>
-      <c r="J6" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H6" s="3" t="n">
         <v>9.99</v>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>BB-FBA</t>
         </is>
       </c>
-      <c r="L6" t="n">
-        <v>7</v>
-      </c>
-      <c r="M6" s="4" t="n">
+      <c r="J6" s="4" t="n">
         <v>0.1545</v>
       </c>
+      <c r="K6" s="3">
+        <f>H6*J6+Z6</f>
+        <v/>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N6" s="3">
-        <f>J6*M6+AD6</f>
+        <f>(H6/1.21)-E6-K6-L6-M6</f>
         <v/>
       </c>
-      <c r="O6" s="3" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="P6" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R6" s="3">
-        <f>(J6/1.21)-E6-N6-O6-P6</f>
+      <c r="O6" s="5">
+        <f>N6/E6</f>
         <v/>
       </c>
-      <c r="S6" s="5">
-        <f>R6/E6</f>
+      <c r="P6" s="5">
+        <f>N6/H6</f>
         <v/>
       </c>
-      <c r="T6" s="5">
-        <f>R6/J6</f>
-        <v/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>VALORAR</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>OK Alm:0 FBA:2</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>AMBIGUO</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Titulo de prueba Beta</t>
+        </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>VALORAR</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>OK Alm:0 FBA:2</t>
+          <t>⚠ DUDOSO</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
+          <t>ninguno pasa el filtro — REVISAR</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>Titulo de prueba Beta</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>⚠ DUDOSO</t>
-        </is>
+          <t>INCOHERENTE: la caja sale a 1.00 €/ud y la unidad suelta del MISMO EAN esta a 5.00 €</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t>Ver ficha ↗</t>
+        </is>
+      </c>
+      <c r="Z6" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="AA6" t="inlineStr">
-        <is>
-          <t>ninguno pasa el filtro — REVISAR</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>INCOHERENTE: la caja sale a 1.00 €/ud y la unidad suelta del MISMO EAN esta a 5.00 €</t>
-        </is>
-      </c>
-      <c r="AC6" s="2" t="inlineStr">
-        <is>
-          <t>Ver ficha ↗</t>
-        </is>
-      </c>
-      <c r="AD6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE6" t="inlineStr">
         <is>
           <t>asumido 21%</t>
         </is>
@@ -1321,70 +1255,70 @@
           <t>IT</t>
         </is>
       </c>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" t="inlineStr">
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" t="inlineStr">
         <is>
           <t>sin datos</t>
         </is>
       </c>
-      <c r="M7" s="4" t="n"/>
+      <c r="J7" s="4" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N7" s="3" t="n"/>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R7" s="3" t="n"/>
-      <c r="S7" s="5" t="n"/>
-      <c r="T7" s="5" t="n"/>
+      <c r="O7" s="5" t="n"/>
+      <c r="P7" s="5" t="n"/>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Sin datos</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>OK Alm:0 FBA:2</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>AMBIGUO</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Titulo de prueba Beta</t>
+        </is>
+      </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Sin datos</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>OK Alm:0 FBA:2</t>
+          <t>⚠ DUDOSO</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
+          <t>ninguno pasa el filtro — REVISAR</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>Titulo de prueba Beta</t>
-        </is>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>⚠ DUDOSO</t>
-        </is>
+          <t>INCOHERENTE: la caja sale a 1.00 €/ud y la unidad suelta del MISMO EAN esta a 5.00 €</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="inlineStr">
+        <is>
+          <t>Ver ficha ↗</t>
+        </is>
+      </c>
+      <c r="Z7" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="AA7" t="inlineStr">
-        <is>
-          <t>ninguno pasa el filtro — REVISAR</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>INCOHERENTE: la caja sale a 1.00 €/ud y la unidad suelta del MISMO EAN esta a 5.00 €</t>
-        </is>
-      </c>
-      <c r="AC7" s="2" t="inlineStr">
-        <is>
-          <t>Ver ficha ↗</t>
-        </is>
-      </c>
-      <c r="AD7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1420,100 +1354,91 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>9000</v>
-      </c>
-      <c r="H8" t="n">
-        <v>18000</v>
-      </c>
-      <c r="I8" t="n">
-        <v>40</v>
-      </c>
-      <c r="J8" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H8" s="3" t="n">
         <v>11.5</v>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>BB-FBA</t>
         </is>
       </c>
-      <c r="L8" t="n">
-        <v>7</v>
-      </c>
-      <c r="M8" s="4" t="n">
+      <c r="J8" s="4" t="n">
         <v>0.1545</v>
       </c>
+      <c r="K8" s="3">
+        <f>H8*J8+Z8</f>
+        <v/>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N8" s="3">
-        <f>J8*M8+AD8</f>
+        <f>(H8/1.2)-E8-K8-L8-M8</f>
         <v/>
       </c>
-      <c r="O8" s="3" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="P8" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R8" s="3">
-        <f>(J8/1.2)-E8-N8-O8-P8</f>
+      <c r="O8" s="5">
+        <f>N8/E8</f>
         <v/>
       </c>
-      <c r="S8" s="5">
-        <f>R8/E8</f>
+      <c r="P8" s="5">
+        <f>N8/H8</f>
         <v/>
       </c>
-      <c r="T8" s="5">
-        <f>R8/J8</f>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>COMPRAR</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>OK Alm:0 FBA:2</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>AMBIGUO</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Titulo de prueba Beta</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>⚠ DUDOSO</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>ninguno pasa el filtro — REVISAR</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>INCOHERENTE: la caja sale a 1.00 €/ud y la unidad suelta del MISMO EAN esta a 5.00 €</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr">
+        <is>
+          <t>Ver ficha ↗</t>
+        </is>
+      </c>
+      <c r="Z8" s="3">
+        <f>L8*0.03</f>
         <v/>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>COMPRAR</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>OK Alm:0 FBA:2</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>AMBIGUO</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>Titulo de prueba Beta</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>⚠ DUDOSO</t>
-        </is>
-      </c>
       <c r="AA8" t="inlineStr">
-        <is>
-          <t>ninguno pasa el filtro — REVISAR</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>INCOHERENTE: la caja sale a 1.00 €/ud y la unidad suelta del MISMO EAN esta a 5.00 €</t>
-        </is>
-      </c>
-      <c r="AC8" s="2" t="inlineStr">
-        <is>
-          <t>Ver ficha ↗</t>
-        </is>
-      </c>
-      <c r="AD8" s="3">
-        <f>O8*0.03</f>
-        <v/>
-      </c>
-      <c r="AE8" t="inlineStr">
         <is>
           <t>general FR 20%</t>
         </is>
@@ -1548,70 +1473,70 @@
           <t>DE</t>
         </is>
       </c>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" t="inlineStr">
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" t="inlineStr">
         <is>
           <t>sin datos</t>
         </is>
       </c>
-      <c r="M9" s="4" t="n"/>
+      <c r="J9" s="4" t="n"/>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
+      <c r="M9" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R9" s="3" t="n"/>
-      <c r="S9" s="5" t="n"/>
-      <c r="T9" s="5" t="n"/>
+      <c r="O9" s="5" t="n"/>
+      <c r="P9" s="5" t="n"/>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Sin datos</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>OK Alm:0 FBA:2</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>AMBIGUO</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Titulo de prueba Beta</t>
+        </is>
+      </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Sin datos</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>OK Alm:0 FBA:2</t>
+          <t>⚠ DUDOSO</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>AMBIGUO</t>
+          <t>ninguno pasa el filtro — REVISAR</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>Titulo de prueba Beta</t>
-        </is>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="Z9" t="inlineStr">
-        <is>
-          <t>⚠ DUDOSO</t>
-        </is>
+          <t>INCOHERENTE: la caja sale a 1.00 €/ud y la unidad suelta del MISMO EAN esta a 5.00 €</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>Ver ficha ↗</t>
+        </is>
+      </c>
+      <c r="Z9" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="AA9" t="inlineStr">
-        <is>
-          <t>ninguno pasa el filtro — REVISAR</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>INCOHERENTE: la caja sale a 1.00 €/ud y la unidad suelta del MISMO EAN esta a 5.00 €</t>
-        </is>
-      </c>
-      <c r="AC9" s="2" t="inlineStr">
-        <is>
-          <t>Ver ficha ↗</t>
-        </is>
-      </c>
-      <c r="AD9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1645,73 +1570,64 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>500</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I10" t="n">
-        <v>40</v>
-      </c>
-      <c r="J10" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H10" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>BB-FBA</t>
         </is>
       </c>
-      <c r="L10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M10" s="4" t="n">
+      <c r="J10" s="4" t="n">
         <v>0.1545</v>
       </c>
-      <c r="N10" s="3">
-        <f>J10*M10+AD10</f>
+      <c r="K10" s="3">
+        <f>H10*J10+Z10</f>
         <v/>
       </c>
-      <c r="O10" s="3" t="n">
+      <c r="L10" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="P10" s="3" t="n">
+      <c r="M10" s="3" t="n">
         <v>0.15</v>
       </c>
-      <c r="R10" s="3" t="n"/>
-      <c r="S10" s="5" t="n"/>
-      <c r="T10" s="5" t="n"/>
-      <c r="U10" t="inlineStr">
+      <c r="N10" s="3" t="n"/>
+      <c r="O10" s="5" t="n"/>
+      <c r="P10" s="5" t="n"/>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>Sin datos</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr">
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>n/d: sin texto que comparar</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>Ver ficha ↗</t>
+        </is>
+      </c>
+      <c r="Z10" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="AA10" t="inlineStr">
-        <is>
-          <t>n/d: sin texto que comparar</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC10" s="2" t="inlineStr">
-        <is>
-          <t>Ver ficha ↗</t>
-        </is>
-      </c>
-      <c r="AD10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE10" t="inlineStr">
         <is>
           <t>asumido 21%</t>
         </is>
@@ -1744,53 +1660,53 @@
           <t>IT</t>
         </is>
       </c>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" t="inlineStr">
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" t="inlineStr">
         <is>
           <t>sin datos</t>
         </is>
       </c>
-      <c r="M11" s="4" t="n"/>
+      <c r="J11" s="4" t="n"/>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
+      <c r="M11" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N11" s="3" t="n"/>
-      <c r="O11" s="3" t="n"/>
-      <c r="P11" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R11" s="3" t="n"/>
-      <c r="S11" s="5" t="n"/>
-      <c r="T11" s="5" t="n"/>
-      <c r="U11" t="inlineStr">
+      <c r="O11" s="5" t="n"/>
+      <c r="P11" s="5" t="n"/>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>Sin datos</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr">
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>n/d: sin texto que comparar</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>Ver ficha ↗</t>
+        </is>
+      </c>
+      <c r="Z11" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="AA11" t="inlineStr">
-        <is>
-          <t>n/d: sin texto que comparar</t>
-        </is>
-      </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC11" s="2" t="inlineStr">
-        <is>
-          <t>Ver ficha ↗</t>
-        </is>
-      </c>
-      <c r="AD11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1823,53 +1739,53 @@
           <t>FR</t>
         </is>
       </c>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" t="inlineStr">
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" t="inlineStr">
         <is>
           <t>sin datos</t>
         </is>
       </c>
-      <c r="M12" s="4" t="n"/>
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N12" s="3" t="n"/>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R12" s="3" t="n"/>
-      <c r="S12" s="5" t="n"/>
-      <c r="T12" s="5" t="n"/>
-      <c r="U12" t="inlineStr">
+      <c r="O12" s="5" t="n"/>
+      <c r="P12" s="5" t="n"/>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>Sin datos</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr">
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>n/d: sin texto que comparar</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>Ver ficha ↗</t>
+        </is>
+      </c>
+      <c r="Z12" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="AA12" t="inlineStr">
-        <is>
-          <t>n/d: sin texto que comparar</t>
-        </is>
-      </c>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC12" s="2" t="inlineStr">
-        <is>
-          <t>Ver ficha ↗</t>
-        </is>
-      </c>
-      <c r="AD12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1902,53 +1818,53 @@
           <t>DE</t>
         </is>
       </c>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" t="inlineStr">
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" t="inlineStr">
         <is>
           <t>sin datos</t>
         </is>
       </c>
-      <c r="M13" s="4" t="n"/>
+      <c r="J13" s="4" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
-      <c r="P13" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R13" s="3" t="n"/>
-      <c r="S13" s="5" t="n"/>
-      <c r="T13" s="5" t="n"/>
-      <c r="U13" t="inlineStr">
+      <c r="O13" s="5" t="n"/>
+      <c r="P13" s="5" t="n"/>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>Sin datos</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr">
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
         <is>
           <t>n/d</t>
         </is>
       </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>n/d: sin texto que comparar</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>Ver ficha ↗</t>
+        </is>
+      </c>
+      <c r="Z13" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="AA13" t="inlineStr">
-        <is>
-          <t>n/d: sin texto que comparar</t>
-        </is>
-      </c>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC13" s="2" t="inlineStr">
-        <is>
-          <t>Ver ficha ↗</t>
-        </is>
-      </c>
-      <c r="AD13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1984,82 +1900,73 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>70000</v>
-      </c>
-      <c r="H14" t="n">
-        <v>140000</v>
-      </c>
-      <c r="I14" t="n">
-        <v>40</v>
-      </c>
-      <c r="J14" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H14" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>BB-FBA</t>
         </is>
       </c>
-      <c r="L14" t="n">
-        <v>7</v>
-      </c>
-      <c r="M14" s="4" t="n">
+      <c r="J14" s="4" t="n">
         <v>0.1545</v>
       </c>
+      <c r="K14" s="3">
+        <f>H14*J14+Z14</f>
+        <v/>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N14" s="3">
-        <f>J14*M14+AD14</f>
+        <f>(H14/1.21)-E14-K14-L14-M14</f>
         <v/>
       </c>
-      <c r="O14" s="3" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="P14" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R14" s="3">
-        <f>(J14/1.21)-E14-N14-O14-P14</f>
+      <c r="O14" s="5">
+        <f>N14/E14</f>
         <v/>
       </c>
-      <c r="S14" s="5">
-        <f>R14/E14</f>
+      <c r="P14" s="5">
+        <f>N14/H14</f>
         <v/>
       </c>
-      <c r="T14" s="5">
-        <f>R14/J14</f>
-        <v/>
-      </c>
-      <c r="U14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>NO COMPRAR</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Titulo Delta</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>Titulo Delta</t>
-        </is>
-      </c>
-      <c r="Z14" t="inlineStr">
-        <is>
           <t>—</t>
         </is>
       </c>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="AA14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AB14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC14" t="inlineStr"/>
-      <c r="AD14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE14" t="inlineStr">
         <is>
           <t>asumido 21%</t>
         </is>
@@ -2095,82 +2002,73 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>60000</v>
-      </c>
-      <c r="H15" t="n">
-        <v>120000</v>
-      </c>
-      <c r="I15" t="n">
-        <v>40</v>
-      </c>
-      <c r="J15" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H15" s="3" t="n">
         <v>8.5</v>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>BB-FBA</t>
         </is>
       </c>
-      <c r="L15" t="n">
-        <v>7</v>
-      </c>
-      <c r="M15" s="4" t="n">
+      <c r="J15" s="4" t="n">
         <v>0.1545</v>
       </c>
+      <c r="K15" s="3">
+        <f>H15*J15+Z15</f>
+        <v/>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N15" s="3">
-        <f>J15*M15+AD15</f>
+        <f>(H15/1.22)-E15-K15-L15-M15</f>
         <v/>
       </c>
-      <c r="O15" s="3" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="P15" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R15" s="3">
-        <f>(J15/1.22)-E15-N15-O15-P15</f>
+      <c r="O15" s="5">
+        <f>N15/E15</f>
         <v/>
       </c>
-      <c r="S15" s="5">
-        <f>R15/E15</f>
+      <c r="P15" s="5">
+        <f>N15/H15</f>
         <v/>
       </c>
-      <c r="T15" s="5">
-        <f>R15/J15</f>
-        <v/>
-      </c>
-      <c r="U15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>NO COMPRAR</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Titulo Delta</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>Titulo Delta</t>
-        </is>
-      </c>
-      <c r="Z15" t="inlineStr">
-        <is>
           <t>—</t>
         </is>
       </c>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="AA15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC15" t="inlineStr"/>
-      <c r="AD15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE15" t="inlineStr">
         <is>
           <t>general IT 22%</t>
         </is>
@@ -2205,53 +2103,53 @@
           <t>FR</t>
         </is>
       </c>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" t="inlineStr">
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" t="inlineStr">
         <is>
           <t>sin datos</t>
         </is>
       </c>
-      <c r="M16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N16" s="3" t="n"/>
-      <c r="O16" s="3" t="n"/>
-      <c r="P16" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R16" s="3" t="n"/>
-      <c r="S16" s="5" t="n"/>
-      <c r="T16" s="5" t="n"/>
-      <c r="U16" t="inlineStr">
+      <c r="O16" s="5" t="n"/>
+      <c r="P16" s="5" t="n"/>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>Sin datos</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Titulo Delta</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>Titulo Delta</t>
-        </is>
-      </c>
-      <c r="Z16" t="inlineStr">
-        <is>
           <t>—</t>
         </is>
       </c>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="AA16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AB16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC16" t="inlineStr"/>
-      <c r="AD16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2286,100 +2184,100 @@
           <t>DE</t>
         </is>
       </c>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" t="inlineStr">
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" t="inlineStr">
         <is>
           <t>sin datos</t>
         </is>
       </c>
-      <c r="M17" s="4" t="n"/>
+      <c r="J17" s="4" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="n">
+        <v>0.15</v>
+      </c>
       <c r="N17" s="3" t="n"/>
-      <c r="O17" s="3" t="n"/>
-      <c r="P17" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R17" s="3" t="n"/>
-      <c r="S17" s="5" t="n"/>
-      <c r="T17" s="5" t="n"/>
-      <c r="U17" t="inlineStr">
+      <c r="O17" s="5" t="n"/>
+      <c r="P17" s="5" t="n"/>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>Sin datos</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Titulo Delta</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>Titulo Delta</t>
-        </is>
-      </c>
-      <c r="Z17" t="inlineStr">
-        <is>
           <t>—</t>
         </is>
       </c>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="AA17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="AB17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC17" t="inlineStr"/>
-      <c r="AD17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="U2:U17">
+  <conditionalFormatting sqref="Q2:Q17">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("NO COMPRAR",U2))</formula>
+      <formula>ISNUMBER(SEARCH("NO COMPRAR",Q2))</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("VALORAR",U2))</formula>
+      <formula>ISNUMBER(SEARCH("VALORAR",Q2))</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("COMPRAR",U2))</formula>
+      <formula>ISNUMBER(SEARCH("COMPRAR",Q2))</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="3" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("Sin datos",U2))</formula>
+      <formula>ISNUMBER(SEARCH("Sin datos",Q2))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T17">
+  <conditionalFormatting sqref="P2:P17">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="4">
       <formula>0.1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y2:Y17">
+  <conditionalFormatting sqref="U2:U17">
     <cfRule type="expression" priority="6" dxfId="0">
-      <formula>ISNUMBER(SEARCH("NO",Y2))</formula>
+      <formula>ISNUMBER(SEARCH("NO",U2))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z2:Z17">
+  <conditionalFormatting sqref="V2:V17">
     <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("DUDOSO",Z2))</formula>
+      <formula>ISNUMBER(SEARCH("DUDOSO",V2))</formula>
     </cfRule>
     <cfRule type="expression" priority="8" dxfId="3" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("n/d",Z2))</formula>
+      <formula>ISNUMBER(SEARCH("n/d",V2))</formula>
     </cfRule>
     <cfRule type="expression" priority="9" dxfId="2" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("OK",Z2))</formula>
+      <formula>ISNUMBER(SEARCH("OK",V2))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB2:AB17">
+  <conditionalFormatting sqref="X2:X17">
     <cfRule type="expression" priority="10" dxfId="0">
-      <formula>ISNUMBER(SEARCH("INCOHERENTE",AB2))</formula>
+      <formula>ISNUMBER(SEARCH("INCOHERENTE",X2))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:AE17">
+  <conditionalFormatting sqref="A2:AA17">
     <cfRule type="expression" priority="11" dxfId="5">
       <formula>ISODD(INT((ROW()-2)/4))</formula>
     </cfRule>
@@ -2390,21 +2288,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y6" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC7" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y7" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC8" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y8" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC9" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y9" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC10" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y10" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC11" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y11" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC12" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y12" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC13" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y13" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId23"/>

</xml_diff>

<commit_message>
Encargo E · «En mi BD» de los escáneres con el stock de verdad (#331)
La columna «En mi BD» del Excel dejaba de leer productos.stock_fba (congelado desde el 22-jul: 155 fichas decían 0 con Amazon teniendo 2.346 uds; Claptrap B0DP7C737P, 0 frente a 18). Ahora los tres escáneres usan una sola función (en_mi_bd.py): FBA = available + fc_transfer de la última foto de inventario_fba sumada por ASIN, con su fecha y «+N en camino»; almacén = productos.stock_moloka, como la v2. Sin dato, raya (nunca 0); foto de más de 2 días, «foto vieja». Arregla también el Excel de novedades, que no pedía stock_moloka. Sin permisos nuevos ni escrituras.

Auditado por Cowork (diff leído salvo test_en_mi_bd.py y el Excel de referencia, por CI).
Fusionado por: sesión «Encargo E», 30-sep-2026.
</commit_message>
<xml_diff>
--- a/excel_referencia_escaner2.xlsx
+++ b/excel_referencia_escaner2.xlsx
@@ -755,7 +755,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>OK Alm:3 FBA:5</t>
+          <t>OK Alm:3 FBA:18 +4 en camino (foto 2026-09-30)</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
@@ -866,7 +866,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>OK Alm:3 FBA:5</t>
+          <t>OK Alm:3 FBA:18 +4 en camino (foto 2026-09-30)</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
@@ -974,7 +974,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>OK Alm:3 FBA:5</t>
+          <t>OK Alm:3 FBA:18 +4 en camino (foto 2026-09-30)</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>OK Alm:3 FBA:5</t>
+          <t>OK Alm:3 FBA:18 +4 en camino (foto 2026-09-30)</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>OK Alm:0 FBA:2</t>
+          <t>OK Alm:0 FBA: — (foto 2026-09-30)</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>OK Alm:0 FBA:2</t>
+          <t>OK Alm:0 FBA: — (foto 2026-09-30)</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>OK Alm:0 FBA:2</t>
+          <t>OK Alm:0 FBA: — (foto 2026-09-30)</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>OK Alm:0 FBA:2</t>
+          <t>OK Alm:0 FBA: — (foto 2026-09-30)</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">

</xml_diff>